<commit_message>
Update spreadsheet via dashboard upload
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erondess\OneDrive - Nokia\Clientes ALU\Meus projetos de desenvolvimento\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nokia-my.sharepoint.com/personal/eron_netto_nokia_com/Documents/Clientes ALU/Meus projetos de desenvolvimento/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B050610-A294-4F14-B9D4-814479D163E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{9B050610-A294-4F14-B9D4-814479D163E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{559E230A-14C2-48FC-93B3-94C0B7B58E10}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{914B9720-525A-4A47-A57F-FCD0334BBABC}"/>
   </bookViews>
@@ -944,10 +944,14 @@
       </c>
       <c r="D3" s="9">
         <f t="shared" ref="D3:D13" si="0">SUM(E3:AQ3)</f>
-        <v>0</v>
-      </c>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
+        <v>19470</v>
+      </c>
+      <c r="E3" s="14">
+        <v>12000</v>
+      </c>
+      <c r="F3" s="14">
+        <v>7470</v>
+      </c>
       <c r="G3" s="14"/>
       <c r="H3" s="14"/>
       <c r="I3" s="14"/>
@@ -996,10 +1000,14 @@
       </c>
       <c r="D4" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
+        <v>21000</v>
+      </c>
+      <c r="E4" s="14">
+        <v>14000</v>
+      </c>
+      <c r="F4" s="14">
+        <v>7000</v>
+      </c>
       <c r="G4" s="14"/>
       <c r="H4" s="14"/>
       <c r="I4" s="14"/>
@@ -1048,10 +1056,14 @@
       </c>
       <c r="D5" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
+        <v>26000</v>
+      </c>
+      <c r="E5" s="14">
+        <v>16000</v>
+      </c>
+      <c r="F5" s="14">
+        <v>10000</v>
+      </c>
       <c r="G5" s="14"/>
       <c r="H5" s="14"/>
       <c r="I5" s="14"/>
@@ -1100,10 +1112,14 @@
       </c>
       <c r="D6" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
+        <v>19000</v>
+      </c>
+      <c r="E6" s="14">
+        <v>8000</v>
+      </c>
+      <c r="F6" s="14">
+        <v>11000</v>
+      </c>
       <c r="G6" s="14"/>
       <c r="H6" s="14"/>
       <c r="I6" s="14"/>
@@ -1152,12 +1168,14 @@
       </c>
       <c r="D7" s="9">
         <f t="shared" si="0"/>
-        <v>7470</v>
+        <v>20470</v>
       </c>
       <c r="E7" s="14">
         <v>7470</v>
       </c>
-      <c r="F7" s="14"/>
+      <c r="F7" s="14">
+        <v>13000</v>
+      </c>
       <c r="G7" s="14"/>
       <c r="H7" s="14"/>
       <c r="I7" s="14"/>
@@ -1206,10 +1224,14 @@
       </c>
       <c r="D8" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
+        <v>7800</v>
+      </c>
+      <c r="E8" s="14">
+        <v>7000</v>
+      </c>
+      <c r="F8" s="14">
+        <v>800</v>
+      </c>
       <c r="G8" s="14"/>
       <c r="H8" s="14"/>
       <c r="I8" s="14"/>
@@ -1258,10 +1280,14 @@
       </c>
       <c r="D9" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
+        <v>22000</v>
+      </c>
+      <c r="E9" s="14">
+        <v>10000</v>
+      </c>
+      <c r="F9" s="14">
+        <v>12000</v>
+      </c>
       <c r="G9" s="14"/>
       <c r="H9" s="14"/>
       <c r="I9" s="14"/>
@@ -1310,10 +1336,14 @@
       </c>
       <c r="D10" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
+        <v>25000</v>
+      </c>
+      <c r="E10" s="14">
+        <v>11000</v>
+      </c>
+      <c r="F10" s="14">
+        <v>14000</v>
+      </c>
       <c r="G10" s="14"/>
       <c r="H10" s="14"/>
       <c r="I10" s="14"/>
@@ -1362,10 +1392,14 @@
       </c>
       <c r="D11" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
+        <v>29000</v>
+      </c>
+      <c r="E11" s="14">
+        <v>13000</v>
+      </c>
+      <c r="F11" s="14">
+        <v>16000</v>
+      </c>
       <c r="G11" s="14"/>
       <c r="H11" s="14"/>
       <c r="I11" s="14"/>
@@ -1414,10 +1448,14 @@
       </c>
       <c r="D12" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
+        <v>8800</v>
+      </c>
+      <c r="E12" s="14">
+        <v>800</v>
+      </c>
+      <c r="F12" s="14">
+        <v>8000</v>
+      </c>
       <c r="G12" s="14"/>
       <c r="H12" s="14"/>
       <c r="I12" s="14"/>
@@ -1464,15 +1502,15 @@
       <c r="C13" s="8"/>
       <c r="D13" s="10">
         <f t="shared" si="0"/>
-        <v>7470</v>
+        <v>198540</v>
       </c>
       <c r="E13" s="18">
         <f t="shared" ref="E13:AQ13" si="1">SUM(E3:E12)</f>
-        <v>7470</v>
+        <v>99270</v>
       </c>
       <c r="F13" s="18">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>99270</v>
       </c>
       <c r="G13" s="18">
         <f t="shared" si="1"/>

</xml_diff>

<commit_message>
Fix merge to preserve spreadsheet structure and remove personal token requirement
- merge_xlsx.py: Use OLD workbook as base, only update cells with new non-zero data
- dashboard_steps.py: Replace GitHub API upload with direct link to GitHub upload page
- Remove all personal token, localStorage, and GitHub API JavaScript code
- Remove unused SheetJS library, toast notifications, and rebuildAll function
- Regenerate index.html

Agent-Logs-Url: https://github.com/eronbfr/Team-8-STC-Nokia/sessions/1c7d7c32-8f15-4852-ad4f-114b2ad0a20e

Co-authored-by: eronbfr <270444003+eronbfr@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -1,191 +1,129 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nokia-my.sharepoint.com/personal/eron_netto_nokia_com/Documents/Clientes ALU/Meus projetos de desenvolvimento/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0000922C-C0BC-4C3F-B2BD-5441BEE16EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{914B9720-525A-4A47-A57F-FCD0334BBABC}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Team 8" sheetId="1" r:id="rId1"/>
+    <sheet name="Team 8" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="12">
-  <si>
-    <t>Wed</t>
-  </si>
-  <si>
-    <t>Thu</t>
-  </si>
-  <si>
-    <t>Fri</t>
-  </si>
-  <si>
-    <t>Sat</t>
-  </si>
-  <si>
-    <t>Sun</t>
-  </si>
-  <si>
-    <t>Mon</t>
-  </si>
-  <si>
-    <t>Tue</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>TOTAL</t>
-  </si>
-  <si>
-    <t>Phone</t>
-  </si>
-  <si>
-    <t>Humberto Silva</t>
-  </si>
-  <si>
-    <t>Total team 8</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="[$-409]d\-mmm;@"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="11">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="16"/>
-      <color rgb="FF242424"/>
       <name val="Nokia Pure Headline Ultra Light"/>
       <family val="2"/>
+      <color rgb="FF242424"/>
+      <sz val="16"/>
     </font>
     <font>
-      <b/>
-      <sz val="16"/>
-      <color rgb="FF242424"/>
       <name val="Nokia Pure Headline Ultra Light"/>
       <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF242424"/>
+      <sz val="16"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF242424"/>
       <name val="Nokia Pure Headline Ultra Light"/>
       <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF242424"/>
+      <sz val="11"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF242424"/>
       <name val="Nokia Pure Headline Ultra Light"/>
       <family val="2"/>
+      <color rgb="FF242424"/>
+      <sz val="11"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FF242424"/>
       <name val="Nokia Pure Headline Ultra Light"/>
       <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF242424"/>
+      <sz val="12"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FF242424"/>
       <name val="Nokia Pure Headline Ultra Light"/>
       <family val="2"/>
+      <color rgb="FF242424"/>
+      <sz val="12"/>
     </font>
     <font>
-      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <sz val="8"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
+        <fgColor theme="7" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
+        <fgColor theme="8" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
+        <fgColor theme="5" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
+        <fgColor theme="9" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -256,94 +194,76 @@
     </border>
   </borders>
   <cellStyleXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="24">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="right" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="right" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="right" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <mruColors>
-      <color rgb="FFCCFFFF"/>
-      <color rgb="FFCCCCFF"/>
-    </mruColors>
-  </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors/>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -642,518 +562,605 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEEA68EC-84D4-45F7-81EB-DA6DEA4C3F46}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:AT7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="3.1796875" customWidth="1"/>
-    <col min="2" max="2" width="24.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.08984375" customWidth="1"/>
-    <col min="4" max="4" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="10.6328125" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="29" width="7.90625" style="2" customWidth="1"/>
-    <col min="30" max="43" width="7.90625" customWidth="1"/>
+    <col width="3.1796875" customWidth="1" min="1" max="1"/>
+    <col width="24.1796875" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="22.08984375" customWidth="1" min="3" max="3"/>
+    <col width="12.453125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="10.6328125" bestFit="1" customWidth="1" style="2" min="5" max="6"/>
+    <col width="7.90625" customWidth="1" style="2" min="7" max="29"/>
+    <col width="7.90625" customWidth="1" min="30" max="43"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:46" x14ac:dyDescent="0.35">
-      <c r="E1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="AC1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="AN1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="AO1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="AP1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="AQ1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="AR1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="AS1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="AT1" s="1" t="s">
-        <v>4</v>
+    <row r="1">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:46" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="B2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="16">
+    <row r="2" ht="15.5" customHeight="1">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E2" s="16" t="n">
         <v>46119</v>
       </c>
-      <c r="F2" s="16">
+      <c r="F2" s="16" t="n">
         <v>46120</v>
       </c>
-      <c r="G2" s="16">
+      <c r="G2" s="16" t="n">
         <v>46121</v>
       </c>
-      <c r="H2" s="16">
+      <c r="H2" s="16" t="n">
         <v>46122</v>
       </c>
-      <c r="I2" s="16">
+      <c r="I2" s="16" t="n">
         <v>46123</v>
       </c>
-      <c r="J2" s="16">
+      <c r="J2" s="16" t="n">
         <v>46124</v>
       </c>
-      <c r="K2" s="16">
+      <c r="K2" s="16" t="n">
         <v>46125</v>
       </c>
-      <c r="L2" s="16">
+      <c r="L2" s="16" t="n">
         <v>46126</v>
       </c>
-      <c r="M2" s="16">
+      <c r="M2" s="16" t="n">
         <v>46127</v>
       </c>
-      <c r="N2" s="16">
+      <c r="N2" s="16" t="n">
         <v>46128</v>
       </c>
-      <c r="O2" s="16">
+      <c r="O2" s="16" t="n">
         <v>46129</v>
       </c>
-      <c r="P2" s="16">
+      <c r="P2" s="16" t="n">
         <v>46130</v>
       </c>
-      <c r="Q2" s="16">
+      <c r="Q2" s="16" t="n">
         <v>46131</v>
       </c>
-      <c r="R2" s="16">
+      <c r="R2" s="16" t="n">
         <v>46132</v>
       </c>
-      <c r="S2" s="16">
+      <c r="S2" s="16" t="n">
         <v>46133</v>
       </c>
-      <c r="T2" s="16">
+      <c r="T2" s="16" t="n">
         <v>46134</v>
       </c>
-      <c r="U2" s="16">
+      <c r="U2" s="16" t="n">
         <v>46135</v>
       </c>
-      <c r="V2" s="16">
+      <c r="V2" s="16" t="n">
         <v>46136</v>
       </c>
-      <c r="W2" s="16">
+      <c r="W2" s="16" t="n">
         <v>46137</v>
       </c>
-      <c r="X2" s="16">
+      <c r="X2" s="16" t="n">
         <v>46138</v>
       </c>
-      <c r="Y2" s="16">
+      <c r="Y2" s="16" t="n">
         <v>46139</v>
       </c>
-      <c r="Z2" s="16">
+      <c r="Z2" s="16" t="n">
         <v>46140</v>
       </c>
-      <c r="AA2" s="16">
+      <c r="AA2" s="16" t="n">
         <v>46141</v>
       </c>
-      <c r="AB2" s="16">
+      <c r="AB2" s="16" t="n">
         <v>46142</v>
       </c>
-      <c r="AC2" s="16">
+      <c r="AC2" s="16" t="n">
         <v>46143</v>
       </c>
-      <c r="AD2" s="16">
+      <c r="AD2" s="16" t="n">
         <v>46144</v>
       </c>
-      <c r="AE2" s="16">
+      <c r="AE2" s="16" t="n">
         <v>46145</v>
       </c>
-      <c r="AF2" s="16">
+      <c r="AF2" s="16" t="n">
         <v>46146</v>
       </c>
-      <c r="AG2" s="16">
+      <c r="AG2" s="16" t="n">
         <v>46147</v>
       </c>
-      <c r="AH2" s="16">
+      <c r="AH2" s="16" t="n">
         <v>46148</v>
       </c>
-      <c r="AI2" s="16">
+      <c r="AI2" s="16" t="n">
         <v>46149</v>
       </c>
-      <c r="AJ2" s="16">
+      <c r="AJ2" s="16" t="n">
         <v>46150</v>
       </c>
-      <c r="AK2" s="16">
+      <c r="AK2" s="16" t="n">
         <v>46151</v>
       </c>
-      <c r="AL2" s="16">
+      <c r="AL2" s="16" t="n">
         <v>46152</v>
       </c>
-      <c r="AM2" s="16">
+      <c r="AM2" s="16" t="n">
         <v>46153</v>
       </c>
-      <c r="AN2" s="16">
+      <c r="AN2" s="16" t="n">
         <v>46154</v>
       </c>
-      <c r="AO2" s="16">
+      <c r="AO2" s="16" t="n">
         <v>46155</v>
       </c>
-      <c r="AP2" s="16">
+      <c r="AP2" s="16" t="n">
         <v>46156</v>
       </c>
-      <c r="AQ2" s="16">
+      <c r="AQ2" s="16" t="n">
         <v>46157</v>
       </c>
     </row>
-    <row r="3" spans="1:46" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="11"/>
-      <c r="B3" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="23">
+    <row r="3" ht="15.5" customHeight="1">
+      <c r="A3" s="11" t="n"/>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Humberto Silva</t>
+        </is>
+      </c>
+      <c r="C3" s="23" t="n">
         <v>5521982184600</v>
       </c>
       <c r="D3" s="9">
-        <f t="shared" ref="D3:D4" si="0">SUM(E3:AQ3)</f>
-        <v>25000</v>
-      </c>
-      <c r="E3" s="14">
+        <f>SUM(E3:AQ3)</f>
+        <v/>
+      </c>
+      <c r="E3" s="14" t="n">
         <v>13000</v>
       </c>
-      <c r="F3" s="14">
+      <c r="F3" s="14" t="n">
         <v>12000</v>
       </c>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
-      <c r="M3" s="15"/>
-      <c r="N3" s="15"/>
-      <c r="O3" s="15"/>
-      <c r="P3" s="15"/>
-      <c r="Q3" s="15"/>
-      <c r="R3" s="20"/>
-      <c r="S3" s="20"/>
-      <c r="T3" s="20"/>
-      <c r="U3" s="20"/>
-      <c r="V3" s="20"/>
-      <c r="W3" s="20"/>
-      <c r="X3" s="20"/>
-      <c r="Y3" s="21"/>
-      <c r="Z3" s="21"/>
-      <c r="AA3" s="21"/>
-      <c r="AB3" s="21"/>
-      <c r="AC3" s="21"/>
-      <c r="AD3" s="21"/>
-      <c r="AE3" s="21"/>
-      <c r="AF3" s="17"/>
-      <c r="AG3" s="22"/>
-      <c r="AH3" s="22"/>
-      <c r="AI3" s="22"/>
-      <c r="AJ3" s="22"/>
-      <c r="AK3" s="22"/>
-      <c r="AL3" s="22"/>
-      <c r="AM3" s="19"/>
-      <c r="AN3" s="19"/>
-      <c r="AO3" s="19"/>
-      <c r="AP3" s="19"/>
-      <c r="AQ3" s="19"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="15" t="n"/>
+      <c r="L3" s="15" t="n"/>
+      <c r="M3" s="15" t="n"/>
+      <c r="N3" s="15" t="n"/>
+      <c r="O3" s="15" t="n"/>
+      <c r="P3" s="15" t="n"/>
+      <c r="Q3" s="15" t="n"/>
+      <c r="R3" s="20" t="n"/>
+      <c r="S3" s="20" t="n"/>
+      <c r="T3" s="20" t="n"/>
+      <c r="U3" s="20" t="n"/>
+      <c r="V3" s="20" t="n"/>
+      <c r="W3" s="20" t="n"/>
+      <c r="X3" s="20" t="n"/>
+      <c r="Y3" s="21" t="n"/>
+      <c r="Z3" s="21" t="n"/>
+      <c r="AA3" s="21" t="n"/>
+      <c r="AB3" s="21" t="n"/>
+      <c r="AC3" s="21" t="n"/>
+      <c r="AD3" s="21" t="n"/>
+      <c r="AE3" s="21" t="n"/>
+      <c r="AF3" s="17" t="n"/>
+      <c r="AG3" s="22" t="n"/>
+      <c r="AH3" s="22" t="n"/>
+      <c r="AI3" s="22" t="n"/>
+      <c r="AJ3" s="22" t="n"/>
+      <c r="AK3" s="22" t="n"/>
+      <c r="AL3" s="22" t="n"/>
+      <c r="AM3" s="19" t="n"/>
+      <c r="AN3" s="19" t="n"/>
+      <c r="AO3" s="19" t="n"/>
+      <c r="AP3" s="19" t="n"/>
+      <c r="AQ3" s="19" t="n"/>
     </row>
-    <row r="4" spans="1:46" s="5" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="13"/>
-      <c r="B4" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="8"/>
+    <row r="4" ht="16" customFormat="1" customHeight="1" s="5" thickBot="1">
+      <c r="A4" s="13" t="n"/>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Total team 8</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="n"/>
       <c r="D4" s="10">
-        <f t="shared" si="0"/>
-        <v>25000</v>
-      </c>
-      <c r="E4" s="18">
-        <f>SUM(E3:E3)</f>
+        <f>SUM(E4:AQ4)</f>
+        <v/>
+      </c>
+      <c r="E4" s="18" t="n">
         <v>13000</v>
       </c>
-      <c r="F4" s="18">
-        <f>SUM(F3:F3)</f>
+      <c r="F4" s="18" t="n">
         <v>12000</v>
       </c>
       <c r="G4" s="18">
         <f>SUM(G3:G3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="H4" s="18">
         <f>SUM(H3:H3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="I4" s="18">
         <f>SUM(I3:I3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="J4" s="18">
         <f>SUM(J3:J3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="K4" s="18">
         <f>SUM(K3:K3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="L4" s="18">
         <f>SUM(L3:L3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="M4" s="18">
         <f>SUM(M3:M3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="N4" s="18">
         <f>SUM(N3:N3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="O4" s="18">
         <f>SUM(O3:O3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="P4" s="18">
         <f>SUM(P3:P3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="Q4" s="18">
         <f>SUM(Q3:Q3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="R4" s="18">
         <f>SUM(R3:R3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="S4" s="18">
         <f>SUM(S3:S3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="T4" s="18">
         <f>SUM(T3:T3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="U4" s="18">
         <f>SUM(U3:U3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="V4" s="18">
         <f>SUM(V3:V3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="W4" s="18">
         <f>SUM(W3:W3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="X4" s="18">
         <f>SUM(X3:X3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="Y4" s="18">
         <f>SUM(Y3:Y3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="Z4" s="18">
         <f>SUM(Z3:Z3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AA4" s="18">
         <f>SUM(AA3:AA3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AB4" s="18">
         <f>SUM(AB3:AB3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AC4" s="18">
         <f>SUM(AC3:AC3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AD4" s="18">
         <f>SUM(AD3:AD3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE4" s="18">
         <f>SUM(AE3:AE3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AF4" s="18">
         <f>SUM(AF3:AF3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AG4" s="18">
         <f>SUM(AG3:AG3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AH4" s="18">
         <f>SUM(AH3:AH3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AI4" s="18">
         <f>SUM(AI3:AI3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AJ4" s="18">
         <f>SUM(AJ3:AJ3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AK4" s="18">
         <f>SUM(AK3:AK3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AL4" s="18">
         <f>SUM(AL3:AL3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AM4" s="18">
         <f>SUM(AM3:AM3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AN4" s="18">
         <f>SUM(AN3:AN3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AO4" s="18">
         <f>SUM(AO3:AO3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AP4" s="18">
         <f>SUM(AP3:AP3)</f>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AQ4" s="18">
         <f>SUM(AQ3:AQ3)</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
-    <row r="5" spans="1:46" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="D5" s="11"/>
+    <row r="5" ht="15" customHeight="1" thickTop="1">
+      <c r="D5" s="11" t="n"/>
     </row>
-    <row r="7" spans="1:46" ht="20.5" x14ac:dyDescent="0.35">
-      <c r="B7" s="12"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="6"/>
+    <row r="6"/>
+    <row r="7" ht="20.5" customHeight="1">
+      <c r="B7" s="12" t="n"/>
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="6" t="n"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3">
-    <sortCondition ref="B3"/>
-  </sortState>
-  <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{5d471751-9675-428d-917b-70f44f9630b0}" enabled="0" method="" siteId="{5d471751-9675-428d-917b-70f44f9630b0}" removed="1"/>
-</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Update step-tracking spreadsheet via dashboard
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nokia-my.sharepoint.com/personal/eron_netto_nokia_com/Documents/Clientes ALU/Meus projetos de desenvolvimento/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{9B050610-A294-4F14-B9D4-814479D163E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AFB414C-8655-4550-8A7C-225EE823227B}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{9B050610-A294-4F14-B9D4-814479D163E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA9B3031-D752-4118-9821-2B080A481C6F}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{914B9720-525A-4A47-A57F-FCD0334BBABC}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="12">
   <si>
     <t>Wed</t>
   </si>
@@ -66,37 +66,10 @@
     <t>Phone</t>
   </si>
   <si>
-    <t>Juan Carloss Moran</t>
-  </si>
-  <si>
-    <t>Humberto Silva</t>
-  </si>
-  <si>
     <t>Total team 8</t>
   </si>
   <si>
-    <t>Rocío Pérez</t>
-  </si>
-  <si>
-    <t>Ruben Salomoni</t>
-  </si>
-  <si>
     <t>Eron Netto</t>
-  </si>
-  <si>
-    <t>Lizandro Ortiz Corzo</t>
-  </si>
-  <si>
-    <t>Alexis Rodriguez</t>
-  </si>
-  <si>
-    <t>Cynthia Vellena</t>
-  </si>
-  <si>
-    <t>Ramiro Campos</t>
-  </si>
-  <si>
-    <t>Jesse Pereira Galvez</t>
   </si>
 </sst>
 </file>
@@ -670,7 +643,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEEA68EC-84D4-45F7-81EB-DA6DEA4C3F46}">
-  <dimension ref="A1:AT16"/>
+  <dimension ref="A1:AT7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="3.1796875" customWidth="1"/>
@@ -941,16 +914,18 @@
     <row r="3" spans="1:46" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="11"/>
       <c r="B3" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C3" s="23">
-        <v>593993955972</v>
+        <v>5521974530828</v>
       </c>
       <c r="D3" s="9">
-        <f t="shared" ref="D3:D13" si="0">SUM(E3:AQ3)</f>
-        <v>0</v>
-      </c>
-      <c r="E3" s="14"/>
+        <f t="shared" ref="D3:D4" si="0">SUM(E3:AQ3)</f>
+        <v>7470</v>
+      </c>
+      <c r="E3" s="14">
+        <v>7470</v>
+      </c>
       <c r="F3" s="14"/>
       <c r="G3" s="14"/>
       <c r="H3" s="14"/>
@@ -990,652 +965,184 @@
       <c r="AP3" s="19"/>
       <c r="AQ3" s="19"/>
     </row>
-    <row r="4" spans="1:46" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="11"/>
-      <c r="B4" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="23">
-        <v>5521982184600</v>
-      </c>
-      <c r="D4" s="9">
+    <row r="4" spans="1:46" s="5" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="13"/>
+      <c r="B4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="8"/>
+      <c r="D4" s="10">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="14"/>
-      <c r="K4" s="15"/>
-      <c r="L4" s="15"/>
-      <c r="M4" s="15"/>
-      <c r="N4" s="15"/>
-      <c r="O4" s="15"/>
-      <c r="P4" s="15"/>
-      <c r="Q4" s="15"/>
-      <c r="R4" s="20"/>
-      <c r="S4" s="20"/>
-      <c r="T4" s="20"/>
-      <c r="U4" s="20"/>
-      <c r="V4" s="20"/>
-      <c r="W4" s="20"/>
-      <c r="X4" s="20"/>
-      <c r="Y4" s="21"/>
-      <c r="Z4" s="21"/>
-      <c r="AA4" s="21"/>
-      <c r="AB4" s="21"/>
-      <c r="AC4" s="21"/>
-      <c r="AD4" s="21"/>
-      <c r="AE4" s="21"/>
-      <c r="AF4" s="17"/>
-      <c r="AG4" s="22"/>
-      <c r="AH4" s="22"/>
-      <c r="AI4" s="22"/>
-      <c r="AJ4" s="22"/>
-      <c r="AK4" s="22"/>
-      <c r="AL4" s="22"/>
-      <c r="AM4" s="19"/>
-      <c r="AN4" s="19"/>
-      <c r="AO4" s="19"/>
-      <c r="AP4" s="19"/>
-      <c r="AQ4" s="19"/>
+        <v>7470</v>
+      </c>
+      <c r="E4" s="18">
+        <f>SUM(E3:E3)</f>
+        <v>7470</v>
+      </c>
+      <c r="F4" s="18">
+        <f>SUM(F3:F3)</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="18">
+        <f>SUM(G3:G3)</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="18">
+        <f>SUM(H3:H3)</f>
+        <v>0</v>
+      </c>
+      <c r="I4" s="18">
+        <f>SUM(I3:I3)</f>
+        <v>0</v>
+      </c>
+      <c r="J4" s="18">
+        <f>SUM(J3:J3)</f>
+        <v>0</v>
+      </c>
+      <c r="K4" s="18">
+        <f>SUM(K3:K3)</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="18">
+        <f>SUM(L3:L3)</f>
+        <v>0</v>
+      </c>
+      <c r="M4" s="18">
+        <f>SUM(M3:M3)</f>
+        <v>0</v>
+      </c>
+      <c r="N4" s="18">
+        <f>SUM(N3:N3)</f>
+        <v>0</v>
+      </c>
+      <c r="O4" s="18">
+        <f>SUM(O3:O3)</f>
+        <v>0</v>
+      </c>
+      <c r="P4" s="18">
+        <f>SUM(P3:P3)</f>
+        <v>0</v>
+      </c>
+      <c r="Q4" s="18">
+        <f>SUM(Q3:Q3)</f>
+        <v>0</v>
+      </c>
+      <c r="R4" s="18">
+        <f>SUM(R3:R3)</f>
+        <v>0</v>
+      </c>
+      <c r="S4" s="18">
+        <f>SUM(S3:S3)</f>
+        <v>0</v>
+      </c>
+      <c r="T4" s="18">
+        <f>SUM(T3:T3)</f>
+        <v>0</v>
+      </c>
+      <c r="U4" s="18">
+        <f>SUM(U3:U3)</f>
+        <v>0</v>
+      </c>
+      <c r="V4" s="18">
+        <f>SUM(V3:V3)</f>
+        <v>0</v>
+      </c>
+      <c r="W4" s="18">
+        <f>SUM(W3:W3)</f>
+        <v>0</v>
+      </c>
+      <c r="X4" s="18">
+        <f>SUM(X3:X3)</f>
+        <v>0</v>
+      </c>
+      <c r="Y4" s="18">
+        <f>SUM(Y3:Y3)</f>
+        <v>0</v>
+      </c>
+      <c r="Z4" s="18">
+        <f>SUM(Z3:Z3)</f>
+        <v>0</v>
+      </c>
+      <c r="AA4" s="18">
+        <f>SUM(AA3:AA3)</f>
+        <v>0</v>
+      </c>
+      <c r="AB4" s="18">
+        <f>SUM(AB3:AB3)</f>
+        <v>0</v>
+      </c>
+      <c r="AC4" s="18">
+        <f>SUM(AC3:AC3)</f>
+        <v>0</v>
+      </c>
+      <c r="AD4" s="18">
+        <f>SUM(AD3:AD3)</f>
+        <v>0</v>
+      </c>
+      <c r="AE4" s="18">
+        <f>SUM(AE3:AE3)</f>
+        <v>0</v>
+      </c>
+      <c r="AF4" s="18">
+        <f>SUM(AF3:AF3)</f>
+        <v>0</v>
+      </c>
+      <c r="AG4" s="18">
+        <f>SUM(AG3:AG3)</f>
+        <v>0</v>
+      </c>
+      <c r="AH4" s="18">
+        <f>SUM(AH3:AH3)</f>
+        <v>0</v>
+      </c>
+      <c r="AI4" s="18">
+        <f>SUM(AI3:AI3)</f>
+        <v>0</v>
+      </c>
+      <c r="AJ4" s="18">
+        <f>SUM(AJ3:AJ3)</f>
+        <v>0</v>
+      </c>
+      <c r="AK4" s="18">
+        <f>SUM(AK3:AK3)</f>
+        <v>0</v>
+      </c>
+      <c r="AL4" s="18">
+        <f>SUM(AL3:AL3)</f>
+        <v>0</v>
+      </c>
+      <c r="AM4" s="18">
+        <f>SUM(AM3:AM3)</f>
+        <v>0</v>
+      </c>
+      <c r="AN4" s="18">
+        <f>SUM(AN3:AN3)</f>
+        <v>0</v>
+      </c>
+      <c r="AO4" s="18">
+        <f>SUM(AO3:AO3)</f>
+        <v>0</v>
+      </c>
+      <c r="AP4" s="18">
+        <f>SUM(AP3:AP3)</f>
+        <v>0</v>
+      </c>
+      <c r="AQ4" s="18">
+        <f>SUM(AQ3:AQ3)</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:46" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="11"/>
-      <c r="B5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="23">
-        <v>525581012681</v>
-      </c>
-      <c r="D5" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
-      <c r="M5" s="15"/>
-      <c r="N5" s="15"/>
-      <c r="O5" s="15"/>
-      <c r="P5" s="15"/>
-      <c r="Q5" s="15"/>
-      <c r="R5" s="20"/>
-      <c r="S5" s="20"/>
-      <c r="T5" s="20"/>
-      <c r="U5" s="20"/>
-      <c r="V5" s="20"/>
-      <c r="W5" s="20"/>
-      <c r="X5" s="20"/>
-      <c r="Y5" s="21"/>
-      <c r="Z5" s="21"/>
-      <c r="AA5" s="21"/>
-      <c r="AB5" s="21"/>
-      <c r="AC5" s="21"/>
-      <c r="AD5" s="21"/>
-      <c r="AE5" s="21"/>
-      <c r="AF5" s="17"/>
-      <c r="AG5" s="22"/>
-      <c r="AH5" s="22"/>
-      <c r="AI5" s="22"/>
-      <c r="AJ5" s="22"/>
-      <c r="AK5" s="22"/>
-      <c r="AL5" s="22"/>
-      <c r="AM5" s="19"/>
-      <c r="AN5" s="19"/>
-      <c r="AO5" s="19"/>
-      <c r="AP5" s="19"/>
-      <c r="AQ5" s="19"/>
+    <row r="5" spans="1:46" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="D5" s="11"/>
     </row>
-    <row r="6" spans="1:46" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="11"/>
-      <c r="B6" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="23">
-        <v>5521993223172</v>
-      </c>
-      <c r="D6" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="15"/>
-      <c r="M6" s="15"/>
-      <c r="N6" s="15"/>
-      <c r="O6" s="15"/>
-      <c r="P6" s="15"/>
-      <c r="Q6" s="15"/>
-      <c r="R6" s="20"/>
-      <c r="S6" s="20"/>
-      <c r="T6" s="20"/>
-      <c r="U6" s="20"/>
-      <c r="V6" s="20"/>
-      <c r="W6" s="20"/>
-      <c r="X6" s="20"/>
-      <c r="Y6" s="21"/>
-      <c r="Z6" s="21"/>
-      <c r="AA6" s="21"/>
-      <c r="AB6" s="21"/>
-      <c r="AC6" s="21"/>
-      <c r="AD6" s="21"/>
-      <c r="AE6" s="21"/>
-      <c r="AF6" s="17"/>
-      <c r="AG6" s="22"/>
-      <c r="AH6" s="22"/>
-      <c r="AI6" s="22"/>
-      <c r="AJ6" s="22"/>
-      <c r="AK6" s="22"/>
-      <c r="AL6" s="22"/>
-      <c r="AM6" s="19"/>
-      <c r="AN6" s="19"/>
-      <c r="AO6" s="19"/>
-      <c r="AP6" s="19"/>
-      <c r="AQ6" s="19"/>
-    </row>
-    <row r="7" spans="1:46" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="11"/>
-      <c r="B7" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="23">
-        <v>5521974530828</v>
-      </c>
-      <c r="D7" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="14"/>
-      <c r="J7" s="14"/>
-      <c r="K7" s="15"/>
-      <c r="L7" s="15"/>
-      <c r="M7" s="15"/>
-      <c r="N7" s="15"/>
-      <c r="O7" s="15"/>
-      <c r="P7" s="15"/>
-      <c r="Q7" s="15"/>
-      <c r="R7" s="20"/>
-      <c r="S7" s="20"/>
-      <c r="T7" s="20"/>
-      <c r="U7" s="20"/>
-      <c r="V7" s="20"/>
-      <c r="W7" s="20"/>
-      <c r="X7" s="20"/>
-      <c r="Y7" s="21"/>
-      <c r="Z7" s="21"/>
-      <c r="AA7" s="21"/>
-      <c r="AB7" s="21"/>
-      <c r="AC7" s="21"/>
-      <c r="AD7" s="21"/>
-      <c r="AE7" s="21"/>
-      <c r="AF7" s="17"/>
-      <c r="AG7" s="22"/>
-      <c r="AH7" s="22"/>
-      <c r="AI7" s="22"/>
-      <c r="AJ7" s="22"/>
-      <c r="AK7" s="22"/>
-      <c r="AL7" s="22"/>
-      <c r="AM7" s="19"/>
-      <c r="AN7" s="19"/>
-      <c r="AO7" s="19"/>
-      <c r="AP7" s="19"/>
-      <c r="AQ7" s="19"/>
-    </row>
-    <row r="8" spans="1:46" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="11"/>
-      <c r="B8" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="23">
-        <v>50256335827</v>
-      </c>
-      <c r="D8" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="15"/>
-      <c r="L8" s="15"/>
-      <c r="M8" s="15"/>
-      <c r="N8" s="15"/>
-      <c r="O8" s="15"/>
-      <c r="P8" s="15"/>
-      <c r="Q8" s="15"/>
-      <c r="R8" s="20"/>
-      <c r="S8" s="20"/>
-      <c r="T8" s="20"/>
-      <c r="U8" s="20"/>
-      <c r="V8" s="20"/>
-      <c r="W8" s="20"/>
-      <c r="X8" s="20"/>
-      <c r="Y8" s="21"/>
-      <c r="Z8" s="21"/>
-      <c r="AA8" s="21"/>
-      <c r="AB8" s="21"/>
-      <c r="AC8" s="21"/>
-      <c r="AD8" s="21"/>
-      <c r="AE8" s="21"/>
-      <c r="AF8" s="17"/>
-      <c r="AG8" s="22"/>
-      <c r="AH8" s="22"/>
-      <c r="AI8" s="22"/>
-      <c r="AJ8" s="22"/>
-      <c r="AK8" s="22"/>
-      <c r="AL8" s="22"/>
-      <c r="AM8" s="19"/>
-      <c r="AN8" s="19"/>
-      <c r="AO8" s="19"/>
-      <c r="AP8" s="19"/>
-      <c r="AQ8" s="19"/>
-    </row>
-    <row r="9" spans="1:46" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="11"/>
-      <c r="B9" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="23">
-        <v>50762003722</v>
-      </c>
-      <c r="D9" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
-      <c r="J9" s="14"/>
-      <c r="K9" s="15"/>
-      <c r="L9" s="15"/>
-      <c r="M9" s="15"/>
-      <c r="N9" s="15"/>
-      <c r="O9" s="15"/>
-      <c r="P9" s="15"/>
-      <c r="Q9" s="15"/>
-      <c r="R9" s="20"/>
-      <c r="S9" s="20"/>
-      <c r="T9" s="20"/>
-      <c r="U9" s="20"/>
-      <c r="V9" s="20"/>
-      <c r="W9" s="20"/>
-      <c r="X9" s="20"/>
-      <c r="Y9" s="21"/>
-      <c r="Z9" s="21"/>
-      <c r="AA9" s="21"/>
-      <c r="AB9" s="21"/>
-      <c r="AC9" s="21"/>
-      <c r="AD9" s="21"/>
-      <c r="AE9" s="21"/>
-      <c r="AF9" s="17"/>
-      <c r="AG9" s="22"/>
-      <c r="AH9" s="22"/>
-      <c r="AI9" s="22"/>
-      <c r="AJ9" s="22"/>
-      <c r="AK9" s="22"/>
-      <c r="AL9" s="22"/>
-      <c r="AM9" s="19"/>
-      <c r="AN9" s="19"/>
-      <c r="AO9" s="19"/>
-      <c r="AP9" s="19"/>
-      <c r="AQ9" s="19"/>
-    </row>
-    <row r="10" spans="1:46" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="11"/>
-      <c r="B10" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10" s="23">
-        <v>51989629245</v>
-      </c>
-      <c r="D10" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="14"/>
-      <c r="J10" s="14"/>
-      <c r="K10" s="15"/>
-      <c r="L10" s="15"/>
-      <c r="M10" s="15"/>
-      <c r="N10" s="15"/>
-      <c r="O10" s="15"/>
-      <c r="P10" s="15"/>
-      <c r="Q10" s="15"/>
-      <c r="R10" s="20"/>
-      <c r="S10" s="20"/>
-      <c r="T10" s="20"/>
-      <c r="U10" s="20"/>
-      <c r="V10" s="20"/>
-      <c r="W10" s="20"/>
-      <c r="X10" s="20"/>
-      <c r="Y10" s="21"/>
-      <c r="Z10" s="21"/>
-      <c r="AA10" s="21"/>
-      <c r="AB10" s="21"/>
-      <c r="AC10" s="21"/>
-      <c r="AD10" s="21"/>
-      <c r="AE10" s="21"/>
-      <c r="AF10" s="17"/>
-      <c r="AG10" s="22"/>
-      <c r="AH10" s="22"/>
-      <c r="AI10" s="22"/>
-      <c r="AJ10" s="22"/>
-      <c r="AK10" s="22"/>
-      <c r="AL10" s="22"/>
-      <c r="AM10" s="19"/>
-      <c r="AN10" s="19"/>
-      <c r="AO10" s="19"/>
-      <c r="AP10" s="19"/>
-      <c r="AQ10" s="19"/>
-    </row>
-    <row r="11" spans="1:46" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="11"/>
-      <c r="B11" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="23">
-        <v>525549447683</v>
-      </c>
-      <c r="D11" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="14"/>
-      <c r="J11" s="14"/>
-      <c r="K11" s="15"/>
-      <c r="L11" s="15"/>
-      <c r="M11" s="15"/>
-      <c r="N11" s="15"/>
-      <c r="O11" s="15"/>
-      <c r="P11" s="15"/>
-      <c r="Q11" s="15"/>
-      <c r="R11" s="20"/>
-      <c r="S11" s="20"/>
-      <c r="T11" s="20"/>
-      <c r="U11" s="20"/>
-      <c r="V11" s="20"/>
-      <c r="W11" s="20"/>
-      <c r="X11" s="20"/>
-      <c r="Y11" s="21"/>
-      <c r="Z11" s="21"/>
-      <c r="AA11" s="21"/>
-      <c r="AB11" s="21"/>
-      <c r="AC11" s="21"/>
-      <c r="AD11" s="21"/>
-      <c r="AE11" s="21"/>
-      <c r="AF11" s="17"/>
-      <c r="AG11" s="22"/>
-      <c r="AH11" s="22"/>
-      <c r="AI11" s="22"/>
-      <c r="AJ11" s="22"/>
-      <c r="AK11" s="22"/>
-      <c r="AL11" s="22"/>
-      <c r="AM11" s="19"/>
-      <c r="AN11" s="19"/>
-      <c r="AO11" s="19"/>
-      <c r="AP11" s="19"/>
-      <c r="AQ11" s="19"/>
-    </row>
-    <row r="12" spans="1:46" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="11"/>
-      <c r="B12" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C12" s="23">
-        <v>5511982355185</v>
-      </c>
-      <c r="D12" s="9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="14"/>
-      <c r="J12" s="14"/>
-      <c r="K12" s="15"/>
-      <c r="L12" s="15"/>
-      <c r="M12" s="15"/>
-      <c r="N12" s="15"/>
-      <c r="O12" s="15"/>
-      <c r="P12" s="15"/>
-      <c r="Q12" s="15"/>
-      <c r="R12" s="20"/>
-      <c r="S12" s="20"/>
-      <c r="T12" s="20"/>
-      <c r="U12" s="20"/>
-      <c r="V12" s="20"/>
-      <c r="W12" s="20"/>
-      <c r="X12" s="20"/>
-      <c r="Y12" s="21"/>
-      <c r="Z12" s="21"/>
-      <c r="AA12" s="21"/>
-      <c r="AB12" s="21"/>
-      <c r="AC12" s="21"/>
-      <c r="AD12" s="21"/>
-      <c r="AE12" s="21"/>
-      <c r="AF12" s="17"/>
-      <c r="AG12" s="22"/>
-      <c r="AH12" s="22"/>
-      <c r="AI12" s="22"/>
-      <c r="AJ12" s="22"/>
-      <c r="AK12" s="22"/>
-      <c r="AL12" s="22"/>
-      <c r="AM12" s="19"/>
-      <c r="AN12" s="19"/>
-      <c r="AO12" s="19"/>
-      <c r="AP12" s="19"/>
-      <c r="AQ12" s="19"/>
-    </row>
-    <row r="13" spans="1:46" s="5" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="13"/>
-      <c r="B13" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E13" s="18">
-        <f t="shared" ref="E13:AQ13" si="1">SUM(E3:E12)</f>
-        <v>0</v>
-      </c>
-      <c r="F13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="L13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="M13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="N13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="O13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="P13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="S13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="T13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="U13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="V13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="W13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="X13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Z13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AA13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AB13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AC13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AD13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AE13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AF13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AG13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AH13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AI13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AJ13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AK13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AL13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AM13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AN13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AO13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AP13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AQ13" s="18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:46" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="D14" s="11"/>
-    </row>
-    <row r="16" spans="1:46" ht="20.5" x14ac:dyDescent="0.35">
-      <c r="B16" s="12"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="6"/>
+    <row r="7" spans="1:46" ht="20.5" x14ac:dyDescent="0.35">
+      <c r="B7" s="12"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="6"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:B12">
-    <sortCondition ref="B3:B12"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3">
+    <sortCondition ref="B3"/>
   </sortState>
   <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>